<commit_message>
linking V0: PoC: Not productive but kinda works. Starting Stances testing/DB/linking V1
</commit_message>
<xml_diff>
--- a/src/entities/extraction/catalogues/keywords.xlsx
+++ b/src/entities/extraction/catalogues/keywords.xlsx
@@ -8,14 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oscarcuellar/ocn/media/kg/kg/src/entities/extraction/catalogues/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0102C941-2F64-E04D-B72D-2474E7361AD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{377C88E4-C169-244D-BB80-8BF16B2FBF1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2540" yWindow="760" windowWidth="29280" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10540" yWindow="3860" windowWidth="29280" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -1297,6 +1310,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N94"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="24.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
added 'enabled' option for keywords/classes, dismissing themes. improved tags prompts
</commit_message>
<xml_diff>
--- a/src/entities/extraction/catalogues/keywords.xlsx
+++ b/src/entities/extraction/catalogues/keywords.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oscarcuellar/ocn/media/kg/kg/src/entities/extraction/catalogues/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CF8DF0A-3588-B54B-8C5F-B800F53644AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0669A72-3524-AD4B-AA4B-039D75868272}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10540" yWindow="3860" windowWidth="29280" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15420" yWindow="4280" windowWidth="29280" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -464,9 +464,6 @@
     <t>protest</t>
   </si>
   <si>
-    <t>"marcha","manifestacion","protesta"</t>
-  </si>
-  <si>
     <t>basura</t>
   </si>
   <si>
@@ -948,6 +945,9 @@
   </si>
   <si>
     <t>enabled</t>
+  </si>
+  <si>
+    <t>"marcha","manifestacion","protesta","protestan"</t>
   </si>
 </sst>
 </file>
@@ -1351,7 +1351,7 @@
         <v>9</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>10</v>
@@ -1385,6 +1385,9 @@
       <c r="J2" t="s">
         <v>19</v>
       </c>
+      <c r="K2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -1405,6 +1408,9 @@
       <c r="J3" t="s">
         <v>19</v>
       </c>
+      <c r="K3" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
@@ -1425,6 +1431,9 @@
       <c r="J4" t="s">
         <v>19</v>
       </c>
+      <c r="K4" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
@@ -1445,6 +1454,9 @@
       <c r="J5" t="s">
         <v>19</v>
       </c>
+      <c r="K5" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
@@ -1465,6 +1477,9 @@
       <c r="J6" t="s">
         <v>19</v>
       </c>
+      <c r="K6" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
@@ -1485,6 +1500,9 @@
       <c r="J7" t="s">
         <v>19</v>
       </c>
+      <c r="K7" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
@@ -1505,6 +1523,9 @@
       <c r="J8" t="s">
         <v>19</v>
       </c>
+      <c r="K8" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
@@ -1528,6 +1549,9 @@
       <c r="J9" t="s">
         <v>19</v>
       </c>
+      <c r="K9" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
@@ -1548,6 +1572,9 @@
       <c r="J10" t="s">
         <v>19</v>
       </c>
+      <c r="K10" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
@@ -1568,6 +1595,9 @@
       <c r="J11" t="s">
         <v>19</v>
       </c>
+      <c r="K11" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
@@ -1588,6 +1618,9 @@
       <c r="J12" t="s">
         <v>19</v>
       </c>
+      <c r="K12" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
@@ -1611,6 +1644,9 @@
       <c r="J13" t="s">
         <v>19</v>
       </c>
+      <c r="K13" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
@@ -1634,6 +1670,9 @@
       <c r="J14" t="s">
         <v>19</v>
       </c>
+      <c r="K14" t="b">
+        <v>1</v>
+      </c>
       <c r="L14" t="s">
         <v>50</v>
       </c>
@@ -1660,6 +1699,9 @@
       <c r="J15" t="s">
         <v>19</v>
       </c>
+      <c r="K15" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
@@ -1683,8 +1725,11 @@
       <c r="J16" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>14</v>
       </c>
@@ -1703,8 +1748,11 @@
       <c r="J17" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>14</v>
       </c>
@@ -1726,8 +1774,11 @@
       <c r="J18" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>64</v>
       </c>
@@ -1746,8 +1797,11 @@
       <c r="J19" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>64</v>
       </c>
@@ -1766,8 +1820,11 @@
       <c r="J20" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>64</v>
       </c>
@@ -1786,8 +1843,11 @@
       <c r="J21" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>64</v>
       </c>
@@ -1806,8 +1866,11 @@
       <c r="J22" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>75</v>
       </c>
@@ -1826,8 +1889,11 @@
       <c r="J23" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K23" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>75</v>
       </c>
@@ -1846,8 +1912,11 @@
       <c r="J24" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>75</v>
       </c>
@@ -1866,8 +1935,11 @@
       <c r="J25" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K25" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>75</v>
       </c>
@@ -1886,8 +1958,11 @@
       <c r="J26" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K26" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>75</v>
       </c>
@@ -1909,8 +1984,11 @@
       <c r="J27" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>64</v>
       </c>
@@ -1929,8 +2007,11 @@
       <c r="J28" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K28" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>64</v>
       </c>
@@ -1949,8 +2030,11 @@
       <c r="J29" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K29" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>64</v>
       </c>
@@ -1969,8 +2053,11 @@
       <c r="J30" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K30" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>64</v>
       </c>
@@ -1989,8 +2076,11 @@
       <c r="J31" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K31" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>64</v>
       </c>
@@ -2009,8 +2099,11 @@
       <c r="J32" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K32" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>75</v>
       </c>
@@ -2029,8 +2122,11 @@
       <c r="J33" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K33" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>75</v>
       </c>
@@ -2044,13 +2140,16 @@
         <v>112</v>
       </c>
       <c r="E34" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="J34" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K34" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>75</v>
       </c>
@@ -2069,8 +2168,11 @@
       <c r="J35" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>75</v>
       </c>
@@ -2089,8 +2191,11 @@
       <c r="J36" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K36" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>117</v>
       </c>
@@ -2109,8 +2214,11 @@
       <c r="J37" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K37" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>117</v>
       </c>
@@ -2129,8 +2237,11 @@
       <c r="J38" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K38" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>117</v>
       </c>
@@ -2149,8 +2260,11 @@
       <c r="J39" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K39" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>117</v>
       </c>
@@ -2169,8 +2283,11 @@
       <c r="J40" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K40" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>117</v>
       </c>
@@ -2189,8 +2306,11 @@
       <c r="J41" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K41" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>117</v>
       </c>
@@ -2209,8 +2329,11 @@
       <c r="J42" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K42" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>117</v>
       </c>
@@ -2229,8 +2352,11 @@
       <c r="J43" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K43" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>64</v>
       </c>
@@ -2249,8 +2375,11 @@
       <c r="J44" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K44" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>75</v>
       </c>
@@ -2264,53 +2393,62 @@
         <v>142</v>
       </c>
       <c r="E45" t="s">
-        <v>143</v>
+        <v>304</v>
       </c>
       <c r="J45" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K45" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>75</v>
       </c>
       <c r="B46" t="s">
+        <v>143</v>
+      </c>
+      <c r="C46" t="s">
+        <v>143</v>
+      </c>
+      <c r="D46" t="s">
         <v>144</v>
       </c>
-      <c r="C46" t="s">
-        <v>144</v>
-      </c>
-      <c r="D46" t="s">
+      <c r="E46" t="s">
         <v>145</v>
       </c>
-      <c r="E46" t="s">
-        <v>146</v>
-      </c>
       <c r="J46" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K46" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>75</v>
       </c>
       <c r="B47" t="s">
+        <v>146</v>
+      </c>
+      <c r="C47" t="s">
+        <v>146</v>
+      </c>
+      <c r="D47" t="s">
         <v>147</v>
       </c>
-      <c r="C47" t="s">
-        <v>147</v>
-      </c>
-      <c r="D47" t="s">
+      <c r="F47" t="s">
         <v>148</v>
       </c>
-      <c r="F47" t="s">
-        <v>149</v>
-      </c>
       <c r="J47" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K47" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>75</v>
       </c>
@@ -2318,16 +2456,19 @@
         <v>76</v>
       </c>
       <c r="C48" t="s">
+        <v>149</v>
+      </c>
+      <c r="D48" t="s">
         <v>150</v>
       </c>
-      <c r="D48" t="s">
+      <c r="E48" t="s">
         <v>151</v>
       </c>
-      <c r="E48" t="s">
-        <v>152</v>
-      </c>
       <c r="J48" t="s">
         <v>19</v>
+      </c>
+      <c r="K48" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.2">
@@ -2338,19 +2479,22 @@
         <v>76</v>
       </c>
       <c r="C49" t="s">
+        <v>152</v>
+      </c>
+      <c r="D49" t="s">
         <v>153</v>
       </c>
-      <c r="D49" t="s">
+      <c r="F49" t="s">
         <v>154</v>
       </c>
-      <c r="F49" t="s">
+      <c r="J49" t="s">
+        <v>19</v>
+      </c>
+      <c r="K49" t="b">
+        <v>1</v>
+      </c>
+      <c r="O49" t="s">
         <v>155</v>
-      </c>
-      <c r="J49" t="s">
-        <v>19</v>
-      </c>
-      <c r="O49" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.2">
@@ -2361,16 +2505,19 @@
         <v>118</v>
       </c>
       <c r="C50" t="s">
+        <v>156</v>
+      </c>
+      <c r="D50" t="s">
         <v>157</v>
       </c>
-      <c r="D50" t="s">
+      <c r="E50" t="s">
         <v>158</v>
       </c>
-      <c r="E50" t="s">
-        <v>159</v>
-      </c>
       <c r="J50" t="s">
         <v>19</v>
+      </c>
+      <c r="K50" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.2">
@@ -2381,912 +2528,1044 @@
         <v>65</v>
       </c>
       <c r="C51" t="s">
+        <v>159</v>
+      </c>
+      <c r="D51" t="s">
         <v>160</v>
       </c>
-      <c r="D51" t="s">
+      <c r="E51" t="s">
         <v>161</v>
       </c>
-      <c r="E51" t="s">
-        <v>162</v>
-      </c>
       <c r="J51" t="s">
         <v>19</v>
+      </c>
+      <c r="K51" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B52" t="s">
         <v>72</v>
       </c>
       <c r="C52" t="s">
+        <v>163</v>
+      </c>
+      <c r="D52" t="s">
         <v>164</v>
       </c>
-      <c r="D52" t="s">
+      <c r="F52" t="s">
         <v>165</v>
       </c>
-      <c r="F52" t="s">
-        <v>166</v>
-      </c>
       <c r="J52" t="s">
         <v>19</v>
+      </c>
+      <c r="K52" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B53" t="s">
         <v>72</v>
       </c>
       <c r="C53" t="s">
+        <v>163</v>
+      </c>
+      <c r="D53" t="s">
         <v>164</v>
       </c>
-      <c r="D53" t="s">
-        <v>165</v>
-      </c>
       <c r="F53" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="J53" t="s">
         <v>19</v>
+      </c>
+      <c r="K53" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B54" t="s">
         <v>72</v>
       </c>
       <c r="C54" t="s">
+        <v>167</v>
+      </c>
+      <c r="D54" t="s">
         <v>168</v>
       </c>
-      <c r="D54" t="s">
+      <c r="F54" t="s">
         <v>169</v>
       </c>
-      <c r="F54" t="s">
-        <v>170</v>
-      </c>
       <c r="J54" t="s">
         <v>19</v>
+      </c>
+      <c r="K54" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B55" t="s">
         <v>72</v>
       </c>
       <c r="C55" t="s">
+        <v>170</v>
+      </c>
+      <c r="D55" t="s">
         <v>171</v>
       </c>
-      <c r="D55" t="s">
+      <c r="F55" t="s">
         <v>172</v>
       </c>
-      <c r="F55" t="s">
-        <v>173</v>
-      </c>
       <c r="J55" t="s">
         <v>19</v>
+      </c>
+      <c r="K55" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B56" t="s">
         <v>72</v>
       </c>
       <c r="C56" t="s">
+        <v>173</v>
+      </c>
+      <c r="D56" t="s">
         <v>174</v>
       </c>
-      <c r="D56" t="s">
+      <c r="F56" t="s">
         <v>175</v>
       </c>
-      <c r="F56" t="s">
-        <v>176</v>
-      </c>
       <c r="J56" t="s">
         <v>19</v>
+      </c>
+      <c r="K56" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B57" t="s">
         <v>89</v>
       </c>
       <c r="C57" t="s">
+        <v>176</v>
+      </c>
+      <c r="D57" t="s">
         <v>177</v>
       </c>
-      <c r="D57" t="s">
+      <c r="F57" t="s">
         <v>178</v>
       </c>
-      <c r="F57" t="s">
-        <v>179</v>
-      </c>
       <c r="J57" t="s">
         <v>19</v>
+      </c>
+      <c r="K57" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="58" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B58" t="s">
         <v>89</v>
       </c>
       <c r="C58" t="s">
+        <v>179</v>
+      </c>
+      <c r="D58" t="s">
         <v>180</v>
       </c>
-      <c r="D58" t="s">
+      <c r="F58" t="s">
         <v>181</v>
       </c>
-      <c r="F58" t="s">
-        <v>182</v>
-      </c>
       <c r="J58" t="s">
         <v>19</v>
+      </c>
+      <c r="K58" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="59" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B59" t="s">
         <v>89</v>
       </c>
       <c r="C59" t="s">
+        <v>182</v>
+      </c>
+      <c r="D59" t="s">
         <v>183</v>
       </c>
-      <c r="D59" t="s">
+      <c r="F59" t="s">
         <v>184</v>
       </c>
-      <c r="F59" t="s">
-        <v>185</v>
-      </c>
       <c r="J59" t="s">
         <v>19</v>
+      </c>
+      <c r="K59" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="60" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B60" t="s">
         <v>89</v>
       </c>
       <c r="C60" t="s">
+        <v>185</v>
+      </c>
+      <c r="D60" t="s">
         <v>186</v>
       </c>
-      <c r="D60" t="s">
+      <c r="F60" t="s">
         <v>187</v>
       </c>
-      <c r="F60" t="s">
-        <v>188</v>
-      </c>
       <c r="J60" t="s">
         <v>19</v>
+      </c>
+      <c r="K60" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B61" t="s">
         <v>89</v>
       </c>
       <c r="C61" t="s">
+        <v>188</v>
+      </c>
+      <c r="D61" t="s">
         <v>189</v>
       </c>
-      <c r="D61" t="s">
+      <c r="F61" t="s">
         <v>190</v>
       </c>
-      <c r="F61" t="s">
-        <v>191</v>
-      </c>
       <c r="J61" t="s">
         <v>19</v>
+      </c>
+      <c r="K61" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="62" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B62" t="s">
         <v>89</v>
       </c>
       <c r="C62" t="s">
+        <v>191</v>
+      </c>
+      <c r="D62" t="s">
         <v>192</v>
       </c>
-      <c r="D62" t="s">
+      <c r="F62" t="s">
         <v>193</v>
       </c>
-      <c r="F62" t="s">
-        <v>194</v>
-      </c>
       <c r="J62" t="s">
         <v>19</v>
+      </c>
+      <c r="K62" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B63" t="s">
+        <v>194</v>
+      </c>
+      <c r="C63" t="s">
         <v>195</v>
       </c>
-      <c r="C63" t="s">
+      <c r="D63" t="s">
         <v>196</v>
       </c>
-      <c r="D63" t="s">
+      <c r="F63" t="s">
         <v>197</v>
       </c>
-      <c r="F63" t="s">
-        <v>198</v>
-      </c>
       <c r="J63" t="s">
         <v>19</v>
+      </c>
+      <c r="K63" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B64" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C64" t="s">
+        <v>198</v>
+      </c>
+      <c r="D64" t="s">
         <v>199</v>
       </c>
-      <c r="D64" t="s">
+      <c r="F64" t="s">
         <v>200</v>
       </c>
-      <c r="F64" t="s">
-        <v>201</v>
-      </c>
       <c r="J64" t="s">
         <v>19</v>
+      </c>
+      <c r="K64" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B65" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C65" t="s">
+        <v>201</v>
+      </c>
+      <c r="D65" t="s">
         <v>202</v>
       </c>
-      <c r="D65" t="s">
+      <c r="F65" t="s">
         <v>203</v>
       </c>
-      <c r="F65" t="s">
-        <v>204</v>
-      </c>
       <c r="J65" t="s">
         <v>19</v>
+      </c>
+      <c r="K65" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B66" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C66" t="s">
+        <v>204</v>
+      </c>
+      <c r="D66" t="s">
         <v>205</v>
       </c>
-      <c r="D66" t="s">
+      <c r="F66" t="s">
         <v>206</v>
       </c>
-      <c r="F66" t="s">
-        <v>207</v>
-      </c>
       <c r="J66" t="s">
         <v>19</v>
+      </c>
+      <c r="K66" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="67" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B67" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C67" t="s">
+        <v>207</v>
+      </c>
+      <c r="D67" t="s">
         <v>208</v>
       </c>
-      <c r="D67" t="s">
+      <c r="F67" t="s">
         <v>209</v>
       </c>
-      <c r="F67" t="s">
-        <v>210</v>
-      </c>
       <c r="J67" t="s">
         <v>19</v>
+      </c>
+      <c r="K67" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B68" t="s">
+        <v>210</v>
+      </c>
+      <c r="C68" t="s">
         <v>211</v>
       </c>
-      <c r="C68" t="s">
+      <c r="D68" t="s">
         <v>212</v>
       </c>
-      <c r="D68" t="s">
-        <v>213</v>
-      </c>
       <c r="F68" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J68" t="s">
         <v>19</v>
+      </c>
+      <c r="K68" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="69" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B69" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C69" t="s">
+        <v>213</v>
+      </c>
+      <c r="D69" t="s">
         <v>214</v>
       </c>
-      <c r="D69" t="s">
-        <v>215</v>
-      </c>
       <c r="F69" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J69" t="s">
         <v>19</v>
+      </c>
+      <c r="K69" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="70" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B70" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C70" t="s">
+        <v>215</v>
+      </c>
+      <c r="D70" t="s">
         <v>216</v>
       </c>
-      <c r="D70" t="s">
+      <c r="F70" t="s">
         <v>217</v>
       </c>
-      <c r="F70" t="s">
-        <v>218</v>
-      </c>
       <c r="J70" t="s">
         <v>19</v>
+      </c>
+      <c r="K70" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="71" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B71" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C71" t="s">
+        <v>218</v>
+      </c>
+      <c r="D71" t="s">
         <v>219</v>
       </c>
-      <c r="D71" t="s">
+      <c r="F71" t="s">
         <v>220</v>
       </c>
-      <c r="F71" t="s">
-        <v>221</v>
-      </c>
       <c r="J71" t="s">
         <v>19</v>
+      </c>
+      <c r="K71" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="72" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B72" t="s">
+        <v>221</v>
+      </c>
+      <c r="C72" t="s">
         <v>222</v>
       </c>
-      <c r="C72" t="s">
+      <c r="D72" t="s">
         <v>223</v>
       </c>
-      <c r="D72" t="s">
+      <c r="F72" t="s">
         <v>224</v>
       </c>
-      <c r="F72" t="s">
-        <v>225</v>
-      </c>
       <c r="J72" t="s">
         <v>19</v>
+      </c>
+      <c r="K72" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="73" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B73" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C73" t="s">
+        <v>225</v>
+      </c>
+      <c r="D73" t="s">
         <v>226</v>
       </c>
-      <c r="D73" t="s">
+      <c r="F73" t="s">
         <v>227</v>
       </c>
-      <c r="F73" t="s">
+      <c r="J73" t="s">
+        <v>19</v>
+      </c>
+      <c r="K73" t="b">
+        <v>0</v>
+      </c>
+      <c r="O73" t="s">
         <v>228</v>
-      </c>
-      <c r="J73" t="s">
-        <v>19</v>
-      </c>
-      <c r="O73" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="74" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B74" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C74" t="s">
+        <v>229</v>
+      </c>
+      <c r="D74" t="s">
         <v>230</v>
       </c>
-      <c r="D74" t="s">
+      <c r="F74" t="s">
         <v>231</v>
       </c>
-      <c r="F74" t="s">
-        <v>232</v>
-      </c>
       <c r="J74" t="s">
         <v>19</v>
       </c>
+      <c r="K74" t="b">
+        <v>0</v>
+      </c>
       <c r="O74" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="75" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B75" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C75" t="s">
+        <v>232</v>
+      </c>
+      <c r="D75" t="s">
         <v>233</v>
       </c>
-      <c r="D75" t="s">
+      <c r="E75" t="s">
         <v>234</v>
       </c>
-      <c r="E75" t="s">
+      <c r="F75" t="s">
         <v>235</v>
       </c>
-      <c r="F75" t="s">
-        <v>236</v>
-      </c>
       <c r="J75" t="s">
         <v>19</v>
       </c>
+      <c r="K75" t="b">
+        <v>0</v>
+      </c>
       <c r="O75" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="76" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B76" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C76" t="s">
+        <v>236</v>
+      </c>
+      <c r="D76" t="s">
         <v>237</v>
       </c>
-      <c r="D76" t="s">
+      <c r="F76" t="s">
         <v>238</v>
       </c>
-      <c r="F76" t="s">
-        <v>239</v>
-      </c>
       <c r="J76" t="s">
         <v>19</v>
       </c>
+      <c r="K76" t="b">
+        <v>0</v>
+      </c>
       <c r="O76" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="77" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B77" t="s">
+        <v>239</v>
+      </c>
+      <c r="C77" t="s">
         <v>240</v>
       </c>
-      <c r="C77" t="s">
+      <c r="D77" t="s">
         <v>241</v>
       </c>
-      <c r="D77" t="s">
+      <c r="F77" t="s">
         <v>242</v>
       </c>
-      <c r="F77" t="s">
-        <v>243</v>
-      </c>
       <c r="J77" t="s">
         <v>19</v>
+      </c>
+      <c r="K77" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="78" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B78" t="s">
+        <v>239</v>
+      </c>
+      <c r="C78" t="s">
         <v>240</v>
       </c>
-      <c r="C78" t="s">
+      <c r="D78" t="s">
         <v>241</v>
       </c>
-      <c r="D78" t="s">
-        <v>242</v>
-      </c>
       <c r="I78" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="J78" t="s">
         <v>19</v>
+      </c>
+      <c r="K78" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="79" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B79" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C79" t="s">
+        <v>244</v>
+      </c>
+      <c r="D79" t="s">
         <v>245</v>
       </c>
-      <c r="D79" t="s">
+      <c r="F79" t="s">
         <v>246</v>
       </c>
-      <c r="F79" t="s">
-        <v>247</v>
-      </c>
       <c r="J79" t="s">
         <v>19</v>
+      </c>
+      <c r="K79" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="80" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B80" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C80" t="s">
+        <v>247</v>
+      </c>
+      <c r="D80" t="s">
         <v>248</v>
       </c>
-      <c r="D80" t="s">
+      <c r="F80" t="s">
         <v>249</v>
       </c>
-      <c r="F80" t="s">
+      <c r="J80" t="s">
+        <v>19</v>
+      </c>
+      <c r="K80" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
+        <v>162</v>
+      </c>
+      <c r="B81" t="s">
+        <v>239</v>
+      </c>
+      <c r="C81" t="s">
         <v>250</v>
       </c>
-      <c r="J80" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A81" t="s">
-        <v>163</v>
-      </c>
-      <c r="B81" t="s">
-        <v>240</v>
-      </c>
-      <c r="C81" t="s">
+      <c r="D81" t="s">
         <v>251</v>
       </c>
-      <c r="D81" t="s">
+      <c r="F81" t="s">
         <v>252</v>
       </c>
-      <c r="F81" t="s">
+      <c r="J81" t="s">
+        <v>19</v>
+      </c>
+      <c r="K81" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>162</v>
+      </c>
+      <c r="B82" t="s">
+        <v>239</v>
+      </c>
+      <c r="C82" t="s">
         <v>253</v>
       </c>
-      <c r="J81" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A82" t="s">
-        <v>163</v>
-      </c>
-      <c r="B82" t="s">
-        <v>240</v>
-      </c>
-      <c r="C82" t="s">
+      <c r="D82" t="s">
         <v>254</v>
       </c>
-      <c r="D82" t="s">
+      <c r="F82" t="s">
         <v>255</v>
       </c>
-      <c r="F82" t="s">
+      <c r="J82" t="s">
+        <v>19</v>
+      </c>
+      <c r="K82" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>162</v>
+      </c>
+      <c r="B83" t="s">
         <v>256</v>
       </c>
-      <c r="J82" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A83" t="s">
-        <v>163</v>
-      </c>
-      <c r="B83" t="s">
+      <c r="C83" t="s">
         <v>257</v>
       </c>
-      <c r="C83" t="s">
+      <c r="D83" t="s">
         <v>258</v>
       </c>
-      <c r="D83" t="s">
+      <c r="F83" t="s">
         <v>259</v>
       </c>
-      <c r="F83" t="s">
+      <c r="J83" t="s">
+        <v>19</v>
+      </c>
+      <c r="K83" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
+        <v>162</v>
+      </c>
+      <c r="B84" t="s">
+        <v>256</v>
+      </c>
+      <c r="C84" t="s">
         <v>260</v>
       </c>
-      <c r="J83" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A84" t="s">
-        <v>163</v>
-      </c>
-      <c r="B84" t="s">
-        <v>257</v>
-      </c>
-      <c r="C84" t="s">
+      <c r="D84" t="s">
         <v>261</v>
       </c>
-      <c r="D84" t="s">
+      <c r="E84" t="s">
         <v>262</v>
       </c>
-      <c r="E84" t="s">
+      <c r="F84" t="s">
         <v>263</v>
       </c>
-      <c r="F84" t="s">
+      <c r="J84" t="s">
+        <v>19</v>
+      </c>
+      <c r="K84" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
+        <v>162</v>
+      </c>
+      <c r="B85" t="s">
+        <v>256</v>
+      </c>
+      <c r="C85" t="s">
         <v>264</v>
       </c>
-      <c r="J84" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A85" t="s">
-        <v>163</v>
-      </c>
-      <c r="B85" t="s">
-        <v>257</v>
-      </c>
-      <c r="C85" t="s">
+      <c r="D85" t="s">
         <v>265</v>
       </c>
-      <c r="D85" t="s">
+      <c r="F85" t="s">
         <v>266</v>
       </c>
-      <c r="F85" t="s">
+      <c r="J85" t="s">
+        <v>19</v>
+      </c>
+      <c r="K85" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
+        <v>162</v>
+      </c>
+      <c r="B86" t="s">
+        <v>256</v>
+      </c>
+      <c r="C86" t="s">
         <v>267</v>
       </c>
-      <c r="J85" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A86" t="s">
-        <v>163</v>
-      </c>
-      <c r="B86" t="s">
-        <v>257</v>
-      </c>
-      <c r="C86" t="s">
+      <c r="D86" t="s">
         <v>268</v>
       </c>
-      <c r="D86" t="s">
+      <c r="F86" t="s">
         <v>269</v>
       </c>
-      <c r="F86" t="s">
+      <c r="J86" t="s">
+        <v>19</v>
+      </c>
+      <c r="K86" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>162</v>
+      </c>
+      <c r="B87" t="s">
+        <v>256</v>
+      </c>
+      <c r="C87" t="s">
         <v>270</v>
       </c>
-      <c r="J86" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A87" t="s">
-        <v>163</v>
-      </c>
-      <c r="B87" t="s">
-        <v>257</v>
-      </c>
-      <c r="C87" t="s">
+      <c r="D87" t="s">
         <v>271</v>
       </c>
-      <c r="D87" t="s">
+      <c r="F87" t="s">
         <v>272</v>
       </c>
-      <c r="F87" t="s">
+      <c r="J87" t="s">
+        <v>19</v>
+      </c>
+      <c r="K87" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
         <v>273</v>
       </c>
-      <c r="J87" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A88" t="s">
+      <c r="B88" t="s">
         <v>274</v>
       </c>
-      <c r="B88" t="s">
+      <c r="C88" t="s">
         <v>275</v>
       </c>
-      <c r="C88" t="s">
+      <c r="D88" t="s">
         <v>276</v>
       </c>
-      <c r="D88" t="s">
+      <c r="E88" t="s">
         <v>277</v>
       </c>
-      <c r="E88" t="s">
+      <c r="F88" t="s">
         <v>278</v>
       </c>
-      <c r="F88" t="s">
+      <c r="J88" t="s">
+        <v>19</v>
+      </c>
+      <c r="K88" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>273</v>
+      </c>
+      <c r="B89" t="s">
+        <v>274</v>
+      </c>
+      <c r="C89" t="s">
+        <v>275</v>
+      </c>
+      <c r="D89" t="s">
+        <v>276</v>
+      </c>
+      <c r="F89" t="s">
         <v>279</v>
       </c>
-      <c r="J88" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A89" t="s">
+      <c r="I89" t="s">
+        <v>280</v>
+      </c>
+      <c r="J89" t="s">
+        <v>19</v>
+      </c>
+      <c r="K89" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
+        <v>273</v>
+      </c>
+      <c r="B90" t="s">
         <v>274</v>
       </c>
-      <c r="B89" t="s">
-        <v>275</v>
-      </c>
-      <c r="C89" t="s">
-        <v>276</v>
-      </c>
-      <c r="D89" t="s">
-        <v>277</v>
-      </c>
-      <c r="F89" t="s">
-        <v>280</v>
-      </c>
-      <c r="I89" t="s">
+      <c r="C90" t="s">
         <v>281</v>
       </c>
-      <c r="J89" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A90" t="s">
+      <c r="D90" t="s">
+        <v>282</v>
+      </c>
+      <c r="E90" t="s">
+        <v>283</v>
+      </c>
+      <c r="F90" t="s">
+        <v>284</v>
+      </c>
+      <c r="J90" t="s">
+        <v>19</v>
+      </c>
+      <c r="K90" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>273</v>
+      </c>
+      <c r="B91" t="s">
         <v>274</v>
       </c>
-      <c r="B90" t="s">
-        <v>275</v>
-      </c>
-      <c r="C90" t="s">
-        <v>282</v>
-      </c>
-      <c r="D90" t="s">
-        <v>283</v>
-      </c>
-      <c r="E90" t="s">
-        <v>284</v>
-      </c>
-      <c r="F90" t="s">
+      <c r="C91" t="s">
         <v>285</v>
       </c>
-      <c r="J90" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A91" t="s">
+      <c r="D91" t="s">
+        <v>286</v>
+      </c>
+      <c r="E91" t="s">
+        <v>287</v>
+      </c>
+      <c r="F91" t="s">
+        <v>288</v>
+      </c>
+      <c r="J91" t="s">
+        <v>19</v>
+      </c>
+      <c r="K91" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>273</v>
+      </c>
+      <c r="B92" t="s">
         <v>274</v>
       </c>
-      <c r="B91" t="s">
-        <v>275</v>
-      </c>
-      <c r="C91" t="s">
-        <v>286</v>
-      </c>
-      <c r="D91" t="s">
-        <v>287</v>
-      </c>
-      <c r="E91" t="s">
-        <v>288</v>
-      </c>
-      <c r="F91" t="s">
+      <c r="C92" t="s">
         <v>289</v>
       </c>
-      <c r="J91" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A92" t="s">
+      <c r="D92" t="s">
+        <v>290</v>
+      </c>
+      <c r="E92" t="s">
+        <v>291</v>
+      </c>
+      <c r="F92" t="s">
+        <v>292</v>
+      </c>
+      <c r="J92" t="s">
+        <v>19</v>
+      </c>
+      <c r="K92" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
+        <v>273</v>
+      </c>
+      <c r="B93" t="s">
         <v>274</v>
       </c>
-      <c r="B92" t="s">
-        <v>275</v>
-      </c>
-      <c r="C92" t="s">
-        <v>290</v>
-      </c>
-      <c r="D92" t="s">
-        <v>291</v>
-      </c>
-      <c r="E92" t="s">
-        <v>292</v>
-      </c>
-      <c r="F92" t="s">
+      <c r="C93" t="s">
         <v>293</v>
       </c>
-      <c r="J92" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A93" t="s">
+      <c r="D93" t="s">
+        <v>294</v>
+      </c>
+      <c r="F93" t="s">
+        <v>295</v>
+      </c>
+      <c r="J93" t="s">
+        <v>19</v>
+      </c>
+      <c r="K93" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
+        <v>273</v>
+      </c>
+      <c r="B94" t="s">
         <v>274</v>
       </c>
-      <c r="B93" t="s">
-        <v>275</v>
-      </c>
-      <c r="C93" t="s">
-        <v>294</v>
-      </c>
-      <c r="D93" t="s">
-        <v>295</v>
-      </c>
-      <c r="F93" t="s">
+      <c r="C94" t="s">
         <v>296</v>
       </c>
-      <c r="J93" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A94" t="s">
-        <v>274</v>
-      </c>
-      <c r="B94" t="s">
-        <v>275</v>
-      </c>
-      <c r="C94" t="s">
+      <c r="D94" t="s">
         <v>297</v>
       </c>
-      <c r="D94" t="s">
+      <c r="E94" t="s">
         <v>298</v>
       </c>
-      <c r="E94" t="s">
+      <c r="F94" t="s">
         <v>299</v>
       </c>
-      <c r="F94" t="s">
-        <v>300</v>
-      </c>
       <c r="J94" t="s">
         <v>19</v>
+      </c>
+      <c r="K94" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
extract tries again when bad LLM responses, water_issue into public infrastructure, turned public infrastructure into event (instead of theme)
</commit_message>
<xml_diff>
--- a/src/entities/extraction/catalogues/keywords.xlsx
+++ b/src/entities/extraction/catalogues/keywords.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oscarcuellar/ocn/media/kg/kg/src/entities/extraction/catalogues/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0669A72-3524-AD4B-AA4B-039D75868272}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{463C27FF-B051-5A4A-9B52-E76D358FD32E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15420" yWindow="4280" windowWidth="29280" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -407,9 +407,6 @@
     <t>crash</t>
   </si>
   <si>
-    <t>"choque","chocar","volcadura"</t>
-  </si>
-  <si>
     <t>explosion</t>
   </si>
   <si>
@@ -509,9 +506,6 @@
     <t>pedestrian_hit</t>
   </si>
   <si>
-    <t>"atropellado","atropellar","atropellamiento","atropello"</t>
-  </si>
-  <si>
     <t>secuestro</t>
   </si>
   <si>
@@ -948,6 +942,12 @@
   </si>
   <si>
     <t>"marcha","manifestacion","protesta","protestan"</t>
+  </si>
+  <si>
+    <t>"choque","chocar","volcadura","impactaron","impacto"</t>
+  </si>
+  <si>
+    <t>"atropellado","atropellar","atropellamiento","atropello","arrolla","arrollo"</t>
   </si>
 </sst>
 </file>
@@ -1351,7 +1351,7 @@
         <v>9</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>10</v>
@@ -2140,7 +2140,7 @@
         <v>112</v>
       </c>
       <c r="E34" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="J34" t="s">
         <v>19</v>
@@ -2232,7 +2232,7 @@
         <v>123</v>
       </c>
       <c r="E38" t="s">
-        <v>124</v>
+        <v>303</v>
       </c>
       <c r="J38" t="s">
         <v>19</v>
@@ -2249,13 +2249,13 @@
         <v>118</v>
       </c>
       <c r="C39" t="s">
+        <v>124</v>
+      </c>
+      <c r="D39" t="s">
+        <v>124</v>
+      </c>
+      <c r="E39" t="s">
         <v>125</v>
-      </c>
-      <c r="D39" t="s">
-        <v>125</v>
-      </c>
-      <c r="E39" t="s">
-        <v>126</v>
       </c>
       <c r="J39" t="s">
         <v>19</v>
@@ -2272,13 +2272,13 @@
         <v>118</v>
       </c>
       <c r="C40" t="s">
+        <v>126</v>
+      </c>
+      <c r="D40" t="s">
         <v>127</v>
       </c>
-      <c r="D40" t="s">
+      <c r="E40" t="s">
         <v>128</v>
-      </c>
-      <c r="E40" t="s">
-        <v>129</v>
       </c>
       <c r="J40" t="s">
         <v>19</v>
@@ -2295,13 +2295,13 @@
         <v>118</v>
       </c>
       <c r="C41" t="s">
+        <v>129</v>
+      </c>
+      <c r="D41" t="s">
         <v>130</v>
       </c>
-      <c r="D41" t="s">
+      <c r="E41" t="s">
         <v>131</v>
-      </c>
-      <c r="E41" t="s">
-        <v>132</v>
       </c>
       <c r="J41" t="s">
         <v>19</v>
@@ -2318,13 +2318,13 @@
         <v>118</v>
       </c>
       <c r="C42" t="s">
+        <v>132</v>
+      </c>
+      <c r="D42" t="s">
         <v>133</v>
       </c>
-      <c r="D42" t="s">
+      <c r="E42" t="s">
         <v>134</v>
-      </c>
-      <c r="E42" t="s">
-        <v>135</v>
       </c>
       <c r="J42" t="s">
         <v>19</v>
@@ -2341,10 +2341,10 @@
         <v>118</v>
       </c>
       <c r="C43" t="s">
+        <v>132</v>
+      </c>
+      <c r="D43" t="s">
         <v>133</v>
-      </c>
-      <c r="D43" t="s">
-        <v>134</v>
       </c>
       <c r="I43" t="s">
         <v>117</v>
@@ -2361,16 +2361,16 @@
         <v>64</v>
       </c>
       <c r="B44" t="s">
+        <v>135</v>
+      </c>
+      <c r="C44" t="s">
         <v>136</v>
       </c>
-      <c r="C44" t="s">
+      <c r="D44" t="s">
         <v>137</v>
       </c>
-      <c r="D44" t="s">
+      <c r="E44" t="s">
         <v>138</v>
-      </c>
-      <c r="E44" t="s">
-        <v>139</v>
       </c>
       <c r="J44" t="s">
         <v>19</v>
@@ -2384,16 +2384,16 @@
         <v>75</v>
       </c>
       <c r="B45" t="s">
+        <v>139</v>
+      </c>
+      <c r="C45" t="s">
         <v>140</v>
       </c>
-      <c r="C45" t="s">
+      <c r="D45" t="s">
         <v>141</v>
       </c>
-      <c r="D45" t="s">
-        <v>142</v>
-      </c>
       <c r="E45" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="J45" t="s">
         <v>19</v>
@@ -2407,16 +2407,16 @@
         <v>75</v>
       </c>
       <c r="B46" t="s">
+        <v>142</v>
+      </c>
+      <c r="C46" t="s">
+        <v>142</v>
+      </c>
+      <c r="D46" t="s">
         <v>143</v>
       </c>
-      <c r="C46" t="s">
-        <v>143</v>
-      </c>
-      <c r="D46" t="s">
+      <c r="E46" t="s">
         <v>144</v>
-      </c>
-      <c r="E46" t="s">
-        <v>145</v>
       </c>
       <c r="J46" t="s">
         <v>19</v>
@@ -2430,16 +2430,16 @@
         <v>75</v>
       </c>
       <c r="B47" t="s">
+        <v>145</v>
+      </c>
+      <c r="C47" t="s">
+        <v>145</v>
+      </c>
+      <c r="D47" t="s">
         <v>146</v>
       </c>
-      <c r="C47" t="s">
-        <v>146</v>
-      </c>
-      <c r="D47" t="s">
+      <c r="F47" t="s">
         <v>147</v>
-      </c>
-      <c r="F47" t="s">
-        <v>148</v>
       </c>
       <c r="J47" t="s">
         <v>19</v>
@@ -2456,13 +2456,13 @@
         <v>76</v>
       </c>
       <c r="C48" t="s">
+        <v>148</v>
+      </c>
+      <c r="D48" t="s">
         <v>149</v>
       </c>
-      <c r="D48" t="s">
+      <c r="E48" t="s">
         <v>150</v>
-      </c>
-      <c r="E48" t="s">
-        <v>151</v>
       </c>
       <c r="J48" t="s">
         <v>19</v>
@@ -2479,22 +2479,22 @@
         <v>76</v>
       </c>
       <c r="C49" t="s">
+        <v>151</v>
+      </c>
+      <c r="D49" t="s">
         <v>152</v>
       </c>
-      <c r="D49" t="s">
+      <c r="F49" t="s">
         <v>153</v>
       </c>
-      <c r="F49" t="s">
+      <c r="J49" t="s">
+        <v>19</v>
+      </c>
+      <c r="K49" t="b">
+        <v>1</v>
+      </c>
+      <c r="O49" t="s">
         <v>154</v>
-      </c>
-      <c r="J49" t="s">
-        <v>19</v>
-      </c>
-      <c r="K49" t="b">
-        <v>1</v>
-      </c>
-      <c r="O49" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.2">
@@ -2505,13 +2505,13 @@
         <v>118</v>
       </c>
       <c r="C50" t="s">
+        <v>155</v>
+      </c>
+      <c r="D50" t="s">
         <v>156</v>
       </c>
-      <c r="D50" t="s">
-        <v>157</v>
-      </c>
       <c r="E50" t="s">
-        <v>158</v>
+        <v>304</v>
       </c>
       <c r="J50" t="s">
         <v>19</v>
@@ -2528,13 +2528,13 @@
         <v>65</v>
       </c>
       <c r="C51" t="s">
+        <v>157</v>
+      </c>
+      <c r="D51" t="s">
+        <v>158</v>
+      </c>
+      <c r="E51" t="s">
         <v>159</v>
-      </c>
-      <c r="D51" t="s">
-        <v>160</v>
-      </c>
-      <c r="E51" t="s">
-        <v>161</v>
       </c>
       <c r="J51" t="s">
         <v>19</v>
@@ -2545,19 +2545,19 @@
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B52" t="s">
         <v>72</v>
       </c>
       <c r="C52" t="s">
+        <v>161</v>
+      </c>
+      <c r="D52" t="s">
+        <v>162</v>
+      </c>
+      <c r="F52" t="s">
         <v>163</v>
-      </c>
-      <c r="D52" t="s">
-        <v>164</v>
-      </c>
-      <c r="F52" t="s">
-        <v>165</v>
       </c>
       <c r="J52" t="s">
         <v>19</v>
@@ -2568,19 +2568,19 @@
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B53" t="s">
         <v>72</v>
       </c>
       <c r="C53" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D53" t="s">
+        <v>162</v>
+      </c>
+      <c r="F53" t="s">
         <v>164</v>
-      </c>
-      <c r="F53" t="s">
-        <v>166</v>
       </c>
       <c r="J53" t="s">
         <v>19</v>
@@ -2591,19 +2591,19 @@
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B54" t="s">
         <v>72</v>
       </c>
       <c r="C54" t="s">
+        <v>165</v>
+      </c>
+      <c r="D54" t="s">
+        <v>166</v>
+      </c>
+      <c r="F54" t="s">
         <v>167</v>
-      </c>
-      <c r="D54" t="s">
-        <v>168</v>
-      </c>
-      <c r="F54" t="s">
-        <v>169</v>
       </c>
       <c r="J54" t="s">
         <v>19</v>
@@ -2614,19 +2614,19 @@
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B55" t="s">
         <v>72</v>
       </c>
       <c r="C55" t="s">
+        <v>168</v>
+      </c>
+      <c r="D55" t="s">
+        <v>169</v>
+      </c>
+      <c r="F55" t="s">
         <v>170</v>
-      </c>
-      <c r="D55" t="s">
-        <v>171</v>
-      </c>
-      <c r="F55" t="s">
-        <v>172</v>
       </c>
       <c r="J55" t="s">
         <v>19</v>
@@ -2637,19 +2637,19 @@
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B56" t="s">
         <v>72</v>
       </c>
       <c r="C56" t="s">
+        <v>171</v>
+      </c>
+      <c r="D56" t="s">
+        <v>172</v>
+      </c>
+      <c r="F56" t="s">
         <v>173</v>
-      </c>
-      <c r="D56" t="s">
-        <v>174</v>
-      </c>
-      <c r="F56" t="s">
-        <v>175</v>
       </c>
       <c r="J56" t="s">
         <v>19</v>
@@ -2660,19 +2660,19 @@
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B57" t="s">
         <v>89</v>
       </c>
       <c r="C57" t="s">
+        <v>174</v>
+      </c>
+      <c r="D57" t="s">
+        <v>175</v>
+      </c>
+      <c r="F57" t="s">
         <v>176</v>
-      </c>
-      <c r="D57" t="s">
-        <v>177</v>
-      </c>
-      <c r="F57" t="s">
-        <v>178</v>
       </c>
       <c r="J57" t="s">
         <v>19</v>
@@ -2683,19 +2683,19 @@
     </row>
     <row r="58" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B58" t="s">
         <v>89</v>
       </c>
       <c r="C58" t="s">
+        <v>177</v>
+      </c>
+      <c r="D58" t="s">
+        <v>178</v>
+      </c>
+      <c r="F58" t="s">
         <v>179</v>
-      </c>
-      <c r="D58" t="s">
-        <v>180</v>
-      </c>
-      <c r="F58" t="s">
-        <v>181</v>
       </c>
       <c r="J58" t="s">
         <v>19</v>
@@ -2706,19 +2706,19 @@
     </row>
     <row r="59" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B59" t="s">
         <v>89</v>
       </c>
       <c r="C59" t="s">
+        <v>180</v>
+      </c>
+      <c r="D59" t="s">
+        <v>181</v>
+      </c>
+      <c r="F59" t="s">
         <v>182</v>
-      </c>
-      <c r="D59" t="s">
-        <v>183</v>
-      </c>
-      <c r="F59" t="s">
-        <v>184</v>
       </c>
       <c r="J59" t="s">
         <v>19</v>
@@ -2729,19 +2729,19 @@
     </row>
     <row r="60" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B60" t="s">
         <v>89</v>
       </c>
       <c r="C60" t="s">
+        <v>183</v>
+      </c>
+      <c r="D60" t="s">
+        <v>184</v>
+      </c>
+      <c r="F60" t="s">
         <v>185</v>
-      </c>
-      <c r="D60" t="s">
-        <v>186</v>
-      </c>
-      <c r="F60" t="s">
-        <v>187</v>
       </c>
       <c r="J60" t="s">
         <v>19</v>
@@ -2752,19 +2752,19 @@
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B61" t="s">
         <v>89</v>
       </c>
       <c r="C61" t="s">
+        <v>186</v>
+      </c>
+      <c r="D61" t="s">
+        <v>187</v>
+      </c>
+      <c r="F61" t="s">
         <v>188</v>
-      </c>
-      <c r="D61" t="s">
-        <v>189</v>
-      </c>
-      <c r="F61" t="s">
-        <v>190</v>
       </c>
       <c r="J61" t="s">
         <v>19</v>
@@ -2775,19 +2775,19 @@
     </row>
     <row r="62" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B62" t="s">
         <v>89</v>
       </c>
       <c r="C62" t="s">
+        <v>189</v>
+      </c>
+      <c r="D62" t="s">
+        <v>190</v>
+      </c>
+      <c r="F62" t="s">
         <v>191</v>
-      </c>
-      <c r="D62" t="s">
-        <v>192</v>
-      </c>
-      <c r="F62" t="s">
-        <v>193</v>
       </c>
       <c r="J62" t="s">
         <v>19</v>
@@ -2798,19 +2798,19 @@
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B63" t="s">
+        <v>192</v>
+      </c>
+      <c r="C63" t="s">
+        <v>193</v>
+      </c>
+      <c r="D63" t="s">
         <v>194</v>
       </c>
-      <c r="C63" t="s">
+      <c r="F63" t="s">
         <v>195</v>
-      </c>
-      <c r="D63" t="s">
-        <v>196</v>
-      </c>
-      <c r="F63" t="s">
-        <v>197</v>
       </c>
       <c r="J63" t="s">
         <v>19</v>
@@ -2821,19 +2821,19 @@
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B64" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C64" t="s">
+        <v>196</v>
+      </c>
+      <c r="D64" t="s">
+        <v>197</v>
+      </c>
+      <c r="F64" t="s">
         <v>198</v>
-      </c>
-      <c r="D64" t="s">
-        <v>199</v>
-      </c>
-      <c r="F64" t="s">
-        <v>200</v>
       </c>
       <c r="J64" t="s">
         <v>19</v>
@@ -2844,19 +2844,19 @@
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B65" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C65" t="s">
+        <v>199</v>
+      </c>
+      <c r="D65" t="s">
+        <v>200</v>
+      </c>
+      <c r="F65" t="s">
         <v>201</v>
-      </c>
-      <c r="D65" t="s">
-        <v>202</v>
-      </c>
-      <c r="F65" t="s">
-        <v>203</v>
       </c>
       <c r="J65" t="s">
         <v>19</v>
@@ -2867,19 +2867,19 @@
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B66" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C66" t="s">
+        <v>202</v>
+      </c>
+      <c r="D66" t="s">
+        <v>203</v>
+      </c>
+      <c r="F66" t="s">
         <v>204</v>
-      </c>
-      <c r="D66" t="s">
-        <v>205</v>
-      </c>
-      <c r="F66" t="s">
-        <v>206</v>
       </c>
       <c r="J66" t="s">
         <v>19</v>
@@ -2890,19 +2890,19 @@
     </row>
     <row r="67" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B67" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C67" t="s">
+        <v>205</v>
+      </c>
+      <c r="D67" t="s">
+        <v>206</v>
+      </c>
+      <c r="F67" t="s">
         <v>207</v>
-      </c>
-      <c r="D67" t="s">
-        <v>208</v>
-      </c>
-      <c r="F67" t="s">
-        <v>209</v>
       </c>
       <c r="J67" t="s">
         <v>19</v>
@@ -2913,19 +2913,19 @@
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B68" t="s">
+        <v>208</v>
+      </c>
+      <c r="C68" t="s">
+        <v>209</v>
+      </c>
+      <c r="D68" t="s">
         <v>210</v>
       </c>
-      <c r="C68" t="s">
-        <v>211</v>
-      </c>
-      <c r="D68" t="s">
-        <v>212</v>
-      </c>
       <c r="F68" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="J68" t="s">
         <v>19</v>
@@ -2936,19 +2936,19 @@
     </row>
     <row r="69" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B69" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C69" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D69" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F69" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="J69" t="s">
         <v>19</v>
@@ -2959,19 +2959,19 @@
     </row>
     <row r="70" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B70" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C70" t="s">
+        <v>213</v>
+      </c>
+      <c r="D70" t="s">
+        <v>214</v>
+      </c>
+      <c r="F70" t="s">
         <v>215</v>
-      </c>
-      <c r="D70" t="s">
-        <v>216</v>
-      </c>
-      <c r="F70" t="s">
-        <v>217</v>
       </c>
       <c r="J70" t="s">
         <v>19</v>
@@ -2982,19 +2982,19 @@
     </row>
     <row r="71" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B71" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C71" t="s">
+        <v>216</v>
+      </c>
+      <c r="D71" t="s">
+        <v>217</v>
+      </c>
+      <c r="F71" t="s">
         <v>218</v>
-      </c>
-      <c r="D71" t="s">
-        <v>219</v>
-      </c>
-      <c r="F71" t="s">
-        <v>220</v>
       </c>
       <c r="J71" t="s">
         <v>19</v>
@@ -3005,19 +3005,19 @@
     </row>
     <row r="72" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B72" t="s">
+        <v>219</v>
+      </c>
+      <c r="C72" t="s">
+        <v>220</v>
+      </c>
+      <c r="D72" t="s">
         <v>221</v>
       </c>
-      <c r="C72" t="s">
+      <c r="F72" t="s">
         <v>222</v>
-      </c>
-      <c r="D72" t="s">
-        <v>223</v>
-      </c>
-      <c r="F72" t="s">
-        <v>224</v>
       </c>
       <c r="J72" t="s">
         <v>19</v>
@@ -3028,46 +3028,46 @@
     </row>
     <row r="73" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B73" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C73" t="s">
+        <v>223</v>
+      </c>
+      <c r="D73" t="s">
+        <v>224</v>
+      </c>
+      <c r="F73" t="s">
         <v>225</v>
       </c>
-      <c r="D73" t="s">
+      <c r="J73" t="s">
+        <v>19</v>
+      </c>
+      <c r="K73" t="b">
+        <v>0</v>
+      </c>
+      <c r="O73" t="s">
         <v>226</v>
-      </c>
-      <c r="F73" t="s">
-        <v>227</v>
-      </c>
-      <c r="J73" t="s">
-        <v>19</v>
-      </c>
-      <c r="K73" t="b">
-        <v>0</v>
-      </c>
-      <c r="O73" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="74" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B74" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C74" t="s">
+        <v>227</v>
+      </c>
+      <c r="D74" t="s">
+        <v>228</v>
+      </c>
+      <c r="F74" t="s">
         <v>229</v>
       </c>
-      <c r="D74" t="s">
-        <v>230</v>
-      </c>
-      <c r="F74" t="s">
-        <v>231</v>
-      </c>
       <c r="J74" t="s">
         <v>19</v>
       </c>
@@ -3075,28 +3075,28 @@
         <v>0</v>
       </c>
       <c r="O74" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="75" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B75" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C75" t="s">
+        <v>230</v>
+      </c>
+      <c r="D75" t="s">
+        <v>231</v>
+      </c>
+      <c r="E75" t="s">
         <v>232</v>
       </c>
-      <c r="D75" t="s">
+      <c r="F75" t="s">
         <v>233</v>
       </c>
-      <c r="E75" t="s">
-        <v>234</v>
-      </c>
-      <c r="F75" t="s">
-        <v>235</v>
-      </c>
       <c r="J75" t="s">
         <v>19</v>
       </c>
@@ -3104,25 +3104,25 @@
         <v>0</v>
       </c>
       <c r="O75" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="76" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B76" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C76" t="s">
+        <v>234</v>
+      </c>
+      <c r="D76" t="s">
+        <v>235</v>
+      </c>
+      <c r="F76" t="s">
         <v>236</v>
       </c>
-      <c r="D76" t="s">
-        <v>237</v>
-      </c>
-      <c r="F76" t="s">
-        <v>238</v>
-      </c>
       <c r="J76" t="s">
         <v>19</v>
       </c>
@@ -3130,24 +3130,24 @@
         <v>0</v>
       </c>
       <c r="O76" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="77" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B77" t="s">
+        <v>237</v>
+      </c>
+      <c r="C77" t="s">
+        <v>238</v>
+      </c>
+      <c r="D77" t="s">
         <v>239</v>
       </c>
-      <c r="C77" t="s">
+      <c r="F77" t="s">
         <v>240</v>
-      </c>
-      <c r="D77" t="s">
-        <v>241</v>
-      </c>
-      <c r="F77" t="s">
-        <v>242</v>
       </c>
       <c r="J77" t="s">
         <v>19</v>
@@ -3158,19 +3158,19 @@
     </row>
     <row r="78" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B78" t="s">
+        <v>237</v>
+      </c>
+      <c r="C78" t="s">
+        <v>238</v>
+      </c>
+      <c r="D78" t="s">
         <v>239</v>
       </c>
-      <c r="C78" t="s">
-        <v>240</v>
-      </c>
-      <c r="D78" t="s">
+      <c r="I78" t="s">
         <v>241</v>
-      </c>
-      <c r="I78" t="s">
-        <v>243</v>
       </c>
       <c r="J78" t="s">
         <v>19</v>
@@ -3181,19 +3181,19 @@
     </row>
     <row r="79" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B79" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C79" t="s">
+        <v>242</v>
+      </c>
+      <c r="D79" t="s">
+        <v>243</v>
+      </c>
+      <c r="F79" t="s">
         <v>244</v>
-      </c>
-      <c r="D79" t="s">
-        <v>245</v>
-      </c>
-      <c r="F79" t="s">
-        <v>246</v>
       </c>
       <c r="J79" t="s">
         <v>19</v>
@@ -3204,19 +3204,19 @@
     </row>
     <row r="80" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B80" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C80" t="s">
+        <v>245</v>
+      </c>
+      <c r="D80" t="s">
+        <v>246</v>
+      </c>
+      <c r="F80" t="s">
         <v>247</v>
-      </c>
-      <c r="D80" t="s">
-        <v>248</v>
-      </c>
-      <c r="F80" t="s">
-        <v>249</v>
       </c>
       <c r="J80" t="s">
         <v>19</v>
@@ -3227,19 +3227,19 @@
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B81" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C81" t="s">
+        <v>248</v>
+      </c>
+      <c r="D81" t="s">
+        <v>249</v>
+      </c>
+      <c r="F81" t="s">
         <v>250</v>
-      </c>
-      <c r="D81" t="s">
-        <v>251</v>
-      </c>
-      <c r="F81" t="s">
-        <v>252</v>
       </c>
       <c r="J81" t="s">
         <v>19</v>
@@ -3250,19 +3250,19 @@
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B82" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C82" t="s">
+        <v>251</v>
+      </c>
+      <c r="D82" t="s">
+        <v>252</v>
+      </c>
+      <c r="F82" t="s">
         <v>253</v>
-      </c>
-      <c r="D82" t="s">
-        <v>254</v>
-      </c>
-      <c r="F82" t="s">
-        <v>255</v>
       </c>
       <c r="J82" t="s">
         <v>19</v>
@@ -3273,19 +3273,19 @@
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B83" t="s">
+        <v>254</v>
+      </c>
+      <c r="C83" t="s">
+        <v>255</v>
+      </c>
+      <c r="D83" t="s">
         <v>256</v>
       </c>
-      <c r="C83" t="s">
+      <c r="F83" t="s">
         <v>257</v>
-      </c>
-      <c r="D83" t="s">
-        <v>258</v>
-      </c>
-      <c r="F83" t="s">
-        <v>259</v>
       </c>
       <c r="J83" t="s">
         <v>19</v>
@@ -3296,22 +3296,22 @@
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B84" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="C84" t="s">
+        <v>258</v>
+      </c>
+      <c r="D84" t="s">
+        <v>259</v>
+      </c>
+      <c r="E84" t="s">
         <v>260</v>
       </c>
-      <c r="D84" t="s">
+      <c r="F84" t="s">
         <v>261</v>
-      </c>
-      <c r="E84" t="s">
-        <v>262</v>
-      </c>
-      <c r="F84" t="s">
-        <v>263</v>
       </c>
       <c r="J84" t="s">
         <v>19</v>
@@ -3322,19 +3322,19 @@
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B85" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="C85" t="s">
+        <v>262</v>
+      </c>
+      <c r="D85" t="s">
+        <v>263</v>
+      </c>
+      <c r="F85" t="s">
         <v>264</v>
-      </c>
-      <c r="D85" t="s">
-        <v>265</v>
-      </c>
-      <c r="F85" t="s">
-        <v>266</v>
       </c>
       <c r="J85" t="s">
         <v>19</v>
@@ -3345,19 +3345,19 @@
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B86" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="C86" t="s">
+        <v>265</v>
+      </c>
+      <c r="D86" t="s">
+        <v>266</v>
+      </c>
+      <c r="F86" t="s">
         <v>267</v>
-      </c>
-      <c r="D86" t="s">
-        <v>268</v>
-      </c>
-      <c r="F86" t="s">
-        <v>269</v>
       </c>
       <c r="J86" t="s">
         <v>19</v>
@@ -3368,19 +3368,19 @@
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B87" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="C87" t="s">
+        <v>268</v>
+      </c>
+      <c r="D87" t="s">
+        <v>269</v>
+      </c>
+      <c r="F87" t="s">
         <v>270</v>
-      </c>
-      <c r="D87" t="s">
-        <v>271</v>
-      </c>
-      <c r="F87" t="s">
-        <v>272</v>
       </c>
       <c r="J87" t="s">
         <v>19</v>
@@ -3391,181 +3391,181 @@
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
+        <v>271</v>
+      </c>
+      <c r="B88" t="s">
+        <v>272</v>
+      </c>
+      <c r="C88" t="s">
         <v>273</v>
       </c>
-      <c r="B88" t="s">
+      <c r="D88" t="s">
         <v>274</v>
       </c>
-      <c r="C88" t="s">
+      <c r="E88" t="s">
         <v>275</v>
       </c>
-      <c r="D88" t="s">
+      <c r="F88" t="s">
         <v>276</v>
       </c>
-      <c r="E88" t="s">
-        <v>277</v>
-      </c>
-      <c r="F88" t="s">
-        <v>278</v>
-      </c>
       <c r="J88" t="s">
         <v>19</v>
       </c>
       <c r="K88" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
+        <v>271</v>
+      </c>
+      <c r="B89" t="s">
+        <v>272</v>
+      </c>
+      <c r="C89" t="s">
         <v>273</v>
       </c>
-      <c r="B89" t="s">
+      <c r="D89" t="s">
         <v>274</v>
       </c>
-      <c r="C89" t="s">
-        <v>275</v>
-      </c>
-      <c r="D89" t="s">
-        <v>276</v>
-      </c>
       <c r="F89" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="I89" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="J89" t="s">
         <v>19</v>
       </c>
       <c r="K89" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B90" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C90" t="s">
+        <v>279</v>
+      </c>
+      <c r="D90" t="s">
+        <v>280</v>
+      </c>
+      <c r="E90" t="s">
         <v>281</v>
       </c>
-      <c r="D90" t="s">
+      <c r="F90" t="s">
         <v>282</v>
       </c>
-      <c r="E90" t="s">
-        <v>283</v>
-      </c>
-      <c r="F90" t="s">
-        <v>284</v>
-      </c>
       <c r="J90" t="s">
         <v>19</v>
       </c>
       <c r="K90" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B91" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C91" t="s">
+        <v>283</v>
+      </c>
+      <c r="D91" t="s">
+        <v>284</v>
+      </c>
+      <c r="E91" t="s">
         <v>285</v>
       </c>
-      <c r="D91" t="s">
+      <c r="F91" t="s">
         <v>286</v>
       </c>
-      <c r="E91" t="s">
-        <v>287</v>
-      </c>
-      <c r="F91" t="s">
-        <v>288</v>
-      </c>
       <c r="J91" t="s">
         <v>19</v>
       </c>
       <c r="K91" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B92" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C92" t="s">
+        <v>287</v>
+      </c>
+      <c r="D92" t="s">
+        <v>288</v>
+      </c>
+      <c r="E92" t="s">
         <v>289</v>
       </c>
-      <c r="D92" t="s">
+      <c r="F92" t="s">
         <v>290</v>
       </c>
-      <c r="E92" t="s">
-        <v>291</v>
-      </c>
-      <c r="F92" t="s">
-        <v>292</v>
-      </c>
       <c r="J92" t="s">
         <v>19</v>
       </c>
       <c r="K92" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B93" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C93" t="s">
+        <v>291</v>
+      </c>
+      <c r="D93" t="s">
+        <v>292</v>
+      </c>
+      <c r="F93" t="s">
         <v>293</v>
       </c>
-      <c r="D93" t="s">
-        <v>294</v>
-      </c>
-      <c r="F93" t="s">
-        <v>295</v>
-      </c>
       <c r="J93" t="s">
         <v>19</v>
       </c>
       <c r="K93" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B94" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C94" t="s">
+        <v>294</v>
+      </c>
+      <c r="D94" t="s">
+        <v>295</v>
+      </c>
+      <c r="E94" t="s">
         <v>296</v>
       </c>
-      <c r="D94" t="s">
+      <c r="F94" t="s">
         <v>297</v>
       </c>
-      <c r="E94" t="s">
-        <v>298</v>
-      </c>
-      <c r="F94" t="s">
-        <v>299</v>
-      </c>
       <c r="J94" t="s">
         <v>19</v>
       </c>
       <c r="K94" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(ontology): concert venue/tour + weather-alert keywords (Bunbury & lluvias misses)
concert: += auditorio, gira. flood: += tormenta; phrases 'alerta
purpura/roja/amarilla', 'corriente(s) de agua'. Applied to live kgdb
ontology_matching_rules rows 1/39 in place (seed script full refresh needs
the sequence owner; xlsx stays the source of truth for the next reseed).

From the 2026-08-08 CDMX social batch review: Bunbury (Auditorio Nacional),
SGIRPC alert posts, and the Topilejo flood report all carried none of the
previous keywords.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013eodLQRAzmesL79k8L4cGx
</commit_message>
<xml_diff>
--- a/src/entities/extraction/catalogues/keywords.xlsx
+++ b/src/entities/extraction/catalogues/keywords.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>"concierto"</t>
+          <t>"concierto","auditorio","gira"</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1914,7 +1914,12 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>"inundacion","inundar","encharcamiento","charco","anegar","tromba","lluvia","aguacero","granizada"</t>
+          <t>"inundacion","inundar","encharcamiento","charco","anegar","tromba","lluvia","aguacero","granizada","tormenta"</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>"alerta purpura","alerta roja","alerta amarilla","corriente de agua","corrientes de agua"</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">

</xml_diff>